<commit_message>
refactor: restructure directories for ease of future implementations
</commit_message>
<xml_diff>
--- a/progress.xlsx
+++ b/progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eugene\Research\gut-pacemaker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97496167-D3E3-4AB1-9711-1606234B88FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB8F1EC-E392-475F-B6E6-417C4F07A914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{FF07EFFA-5070-42E1-91C3-AF06B4048632}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{FF07EFFA-5070-42E1-91C3-AF06B4048632}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress" sheetId="1" r:id="rId1"/>
@@ -638,9 +638,6 @@
     <t>Finalizing</t>
   </si>
   <si>
-    <t>UART</t>
-  </si>
-  <si>
     <t>Separate Pacemaker and GES</t>
   </si>
   <si>
@@ -654,6 +651,9 @@
   </si>
   <si>
     <t>The TCP communication of the gut model and the pacemaker will not be possible eventually on FlexPRET. Transitioning from TCP to UART at this stage and then testing on DE1SoC's HPS(Hard Processor System)'s bare metal mode will make the migration to FlexPRET easier, thus seems to be a nessesary process. I plan use virtual UART port pairing to simulate this within PC, then test on the board.</t>
+  </si>
+  <si>
+    <t>Create UART driver</t>
   </si>
 </sst>
 </file>
@@ -882,35 +882,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1318,7 +1318,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DA6F03D-76AC-4C98-896C-92FC84817ECF}">
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.7265625" style="2" customWidth="1"/>
@@ -1374,7 +1374,7 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="27" t="s">
         <v>82</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -1399,11 +1399,11 @@
       <c r="K3" s="5"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="33"/>
-      <c r="B4" s="28" t="s">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="29" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -1424,9 +1424,9 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="33"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
       <c r="D5" s="5" t="s">
         <v>40</v>
       </c>
@@ -1445,9 +1445,9 @@
       <c r="K5" s="5"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" s="33"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
       <c r="D6" s="5" t="s">
         <v>25</v>
       </c>
@@ -1466,9 +1466,9 @@
       <c r="K6" s="5"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="33"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28" t="s">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29" t="s">
         <v>26</v>
       </c>
       <c r="D7" s="5" t="s">
@@ -1491,9 +1491,9 @@
       <c r="K7" s="5"/>
     </row>
     <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="33"/>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
       <c r="D8" s="5" t="s">
         <v>28</v>
       </c>
@@ -1516,11 +1516,11 @@
       <c r="K8" s="5"/>
     </row>
     <row r="9" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="33"/>
-      <c r="B9" s="28" t="s">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="31" t="s">
         <v>57</v>
       </c>
       <c r="D9" s="5" t="s">
@@ -1549,9 +1549,9 @@
       </c>
     </row>
     <row r="10" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="33"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="26"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="32"/>
       <c r="D10" s="5" t="s">
         <v>5</v>
       </c>
@@ -1578,11 +1578,11 @@
       </c>
     </row>
     <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="33"/>
-      <c r="B11" s="28" t="s">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="31" t="s">
         <v>58</v>
       </c>
       <c r="D11" s="5" t="s">
@@ -1611,9 +1611,9 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="33"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="25"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="33"/>
       <c r="D12" s="5" t="s">
         <v>53</v>
       </c>
@@ -1632,9 +1632,9 @@
       <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="33"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="26"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="32"/>
       <c r="D13" s="5" t="s">
         <v>9</v>
       </c>
@@ -1661,11 +1661,11 @@
       </c>
     </row>
     <row r="14" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="33"/>
+      <c r="A14" s="28"/>
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="31" t="s">
         <v>13</v>
       </c>
       <c r="D14" s="5" t="s">
@@ -1692,11 +1692,11 @@
       <c r="K14" s="5"/>
     </row>
     <row r="15" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="33"/>
+      <c r="A15" s="28"/>
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="26"/>
+      <c r="C15" s="32"/>
       <c r="D15" s="5" t="s">
         <v>16</v>
       </c>
@@ -1721,7 +1721,7 @@
       <c r="K15" s="5"/>
     </row>
     <row r="16" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A16" s="33"/>
+      <c r="A16" s="28"/>
       <c r="B16" s="5" t="s">
         <v>43</v>
       </c>
@@ -1746,7 +1746,7 @@
       <c r="K16" s="5"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="24" t="s">
         <v>75</v>
       </c>
       <c r="B17" s="22" t="s">
@@ -1773,7 +1773,7 @@
       <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A18" s="30"/>
+      <c r="A18" s="25"/>
       <c r="B18" s="23"/>
       <c r="C18" s="5" t="s">
         <v>92</v>
@@ -1798,7 +1798,7 @@
       </c>
     </row>
     <row r="19" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A19" s="30"/>
+      <c r="A19" s="25"/>
       <c r="B19" s="19" t="s">
         <v>77</v>
       </c>
@@ -1825,8 +1825,8 @@
       </c>
     </row>
     <row r="20" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A20" s="30"/>
-      <c r="B20" s="28" t="s">
+      <c r="A20" s="25"/>
+      <c r="B20" s="29" t="s">
         <v>95</v>
       </c>
       <c r="C20" s="5" t="s">
@@ -1848,8 +1848,8 @@
       <c r="K20" s="5"/>
     </row>
     <row r="21" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="30"/>
-      <c r="B21" s="28"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="29"/>
       <c r="C21" s="5" t="s">
         <v>97</v>
       </c>
@@ -1871,7 +1871,7 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="30"/>
+      <c r="A22" s="25"/>
       <c r="B22" s="22" t="s">
         <v>103</v>
       </c>
@@ -1894,8 +1894,8 @@
       <c r="K22" s="5"/>
     </row>
     <row r="23" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="30"/>
-      <c r="B23" s="27"/>
+      <c r="A23" s="25"/>
+      <c r="B23" s="30"/>
       <c r="C23" s="5" t="s">
         <v>105</v>
       </c>
@@ -1915,8 +1915,8 @@
       <c r="K23" s="5"/>
     </row>
     <row r="24" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A24" s="30"/>
-      <c r="B24" s="27"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="30"/>
       <c r="C24" s="5" t="s">
         <v>106</v>
       </c>
@@ -1936,7 +1936,7 @@
       <c r="K24" s="5"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A25" s="30"/>
+      <c r="A25" s="25"/>
       <c r="B25" s="23"/>
       <c r="C25" s="5" t="s">
         <v>107</v>
@@ -1955,7 +1955,7 @@
       <c r="K25" s="5"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A26" s="31"/>
+      <c r="A26" s="26"/>
       <c r="B26" s="5" t="s">
         <v>78</v>
       </c>
@@ -1980,7 +1980,7 @@
       </c>
     </row>
     <row r="27" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A27" s="24" t="s">
+      <c r="A27" s="31" t="s">
         <v>79</v>
       </c>
       <c r="B27" s="5" t="s">
@@ -2005,7 +2005,7 @@
       <c r="K27" s="5"/>
     </row>
     <row r="28" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" s="25"/>
+      <c r="A28" s="33"/>
       <c r="B28" s="5" t="s">
         <v>80</v>
       </c>
@@ -2028,7 +2028,7 @@
       <c r="K28" s="5"/>
     </row>
     <row r="29" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A29" s="25"/>
+      <c r="A29" s="33"/>
       <c r="B29" s="5" t="s">
         <v>81</v>
       </c>
@@ -2051,7 +2051,7 @@
       <c r="K29" s="5"/>
     </row>
     <row r="30" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A30" s="25"/>
+      <c r="A30" s="33"/>
       <c r="B30" s="5" t="s">
         <v>84</v>
       </c>
@@ -2074,12 +2074,12 @@
       <c r="K30" s="5"/>
     </row>
     <row r="31" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="25"/>
+      <c r="A31" s="33"/>
       <c r="B31" s="22" t="s">
         <v>132</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D31" s="5"/>
       <c r="E31" s="5"/>
@@ -2095,10 +2095,10 @@
       <c r="K31" s="5"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A32" s="25"/>
+      <c r="A32" s="33"/>
       <c r="B32" s="23"/>
       <c r="C32" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
@@ -2114,7 +2114,7 @@
       <c r="K32" s="5"/>
     </row>
     <row r="33" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A33" s="25"/>
+      <c r="A33" s="33"/>
       <c r="B33" s="5" t="s">
         <v>136</v>
       </c>
@@ -2132,112 +2132,108 @@
         <v>138</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="44.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="25"/>
-      <c r="B34" s="22" t="s">
-        <v>137</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>92</v>
-      </c>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" s="33"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12"/>
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
       <c r="F34" s="5"/>
-      <c r="G34" s="11">
-        <v>45845</v>
-      </c>
+      <c r="G34" s="11"/>
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
       <c r="J34" s="4"/>
-      <c r="K34" s="22" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A35" s="25"/>
-      <c r="B35" s="27"/>
-      <c r="C35" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>146</v>
-      </c>
+      <c r="K34" s="12"/>
+    </row>
+    <row r="35" spans="1:11" ht="44.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="33"/>
+      <c r="B35" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D35" s="5"/>
       <c r="E35" s="5"/>
       <c r="F35" s="5"/>
       <c r="G35" s="11">
-        <v>45852</v>
+        <v>45845</v>
       </c>
       <c r="H35" s="11"/>
       <c r="I35" s="11"/>
       <c r="J35" s="4"/>
-      <c r="K35" s="27"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A36" s="26"/>
-      <c r="B36" s="23"/>
-      <c r="C36" s="23"/>
+      <c r="K35" s="22" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A36" s="33"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="22" t="s">
+        <v>144</v>
+      </c>
       <c r="D36" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E36" s="5"/>
       <c r="F36" s="5"/>
       <c r="G36" s="11">
-        <v>45859</v>
+        <v>45852</v>
       </c>
       <c r="H36" s="11"/>
       <c r="I36" s="11"/>
       <c r="J36" s="4"/>
-      <c r="K36" s="23"/>
-    </row>
-    <row r="37" spans="1:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="B37" s="22" t="s">
-        <v>133</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="D37" s="5"/>
+      <c r="K36" s="30"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A37" s="32"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="5" t="s">
+        <v>146</v>
+      </c>
       <c r="E37" s="5"/>
       <c r="F37" s="5"/>
       <c r="G37" s="11">
-        <v>45866</v>
+        <v>45859</v>
       </c>
       <c r="H37" s="11"/>
       <c r="I37" s="11"/>
       <c r="J37" s="4"/>
-      <c r="K37" s="5"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A38" s="25"/>
-      <c r="B38" s="27"/>
+      <c r="K37" s="23"/>
+    </row>
+    <row r="38" spans="1:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" s="22" t="s">
+        <v>133</v>
+      </c>
       <c r="C38" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
       <c r="F38" s="5"/>
       <c r="G38" s="11">
-        <v>45873</v>
+        <v>45866</v>
       </c>
       <c r="H38" s="11"/>
       <c r="I38" s="11"/>
       <c r="J38" s="4"/>
       <c r="K38" s="5"/>
     </row>
-    <row r="39" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A39" s="25"/>
-      <c r="B39" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C39" s="5"/>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39" s="33"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="5" t="s">
+        <v>135</v>
+      </c>
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
       <c r="F39" s="5"/>
       <c r="G39" s="11">
-        <v>45880</v>
+        <v>45873</v>
       </c>
       <c r="H39" s="11"/>
       <c r="I39" s="11"/>
@@ -2245,110 +2241,130 @@
       <c r="K39" s="5"/>
     </row>
     <row r="40" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A40" s="25"/>
+      <c r="A40" s="33"/>
       <c r="B40" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
       <c r="F40" s="5"/>
       <c r="G40" s="11">
-        <v>45887</v>
+        <v>45880</v>
       </c>
       <c r="H40" s="11"/>
       <c r="I40" s="11"/>
       <c r="J40" s="4"/>
       <c r="K40" s="5"/>
     </row>
-    <row r="41" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A41" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B41" s="5"/>
+    <row r="41" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A41" s="33"/>
+      <c r="B41" s="5" t="s">
+        <v>86</v>
+      </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
       <c r="F41" s="5"/>
       <c r="G41" s="11">
-        <v>45894</v>
-      </c>
-      <c r="H41" s="11">
-        <v>45900</v>
-      </c>
+        <v>45887</v>
+      </c>
+      <c r="H41" s="11"/>
       <c r="I41" s="11"/>
       <c r="J41" s="4"/>
       <c r="K41" s="5"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A42" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>141</v>
-      </c>
+    <row r="42" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A42" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B42" s="5"/>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
       <c r="F42" s="5"/>
       <c r="G42" s="11">
-        <v>45901</v>
-      </c>
-      <c r="H42" s="11"/>
+        <v>45894</v>
+      </c>
+      <c r="H42" s="11">
+        <v>45900</v>
+      </c>
       <c r="I42" s="11"/>
       <c r="J42" s="4"/>
       <c r="K42" s="5"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A43" s="27"/>
-      <c r="B43" s="5"/>
+      <c r="A43" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>141</v>
+      </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="5"/>
       <c r="F43" s="5"/>
-      <c r="G43" s="11"/>
+      <c r="G43" s="11">
+        <v>45901</v>
+      </c>
       <c r="H43" s="11"/>
       <c r="I43" s="11"/>
       <c r="J43" s="4"/>
       <c r="K43" s="5"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A44" s="23"/>
-      <c r="B44" s="5" t="s">
-        <v>142</v>
-      </c>
+      <c r="A44" s="30"/>
+      <c r="B44" s="5"/>
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
       <c r="E44" s="5"/>
       <c r="F44" s="5"/>
-      <c r="G44" s="11">
-        <v>45929</v>
-      </c>
+      <c r="G44" s="11"/>
       <c r="H44" s="11"/>
       <c r="I44" s="11"/>
       <c r="J44" s="4"/>
       <c r="K44" s="5"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
+      <c r="A45" s="23"/>
+      <c r="B45" s="5" t="s">
+        <v>142</v>
+      </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
-      <c r="G45" s="11"/>
+      <c r="G45" s="11">
+        <v>45929</v>
+      </c>
       <c r="H45" s="11"/>
       <c r="I45" s="11"/>
       <c r="J45" s="4"/>
       <c r="K45" s="5"/>
     </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A46" s="5"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="11"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="11"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="5"/>
+    </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="A17:A26"/>
-    <mergeCell ref="A3:A16"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="A27:A37"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="K35:K37"/>
+    <mergeCell ref="A43:A45"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B38:B39"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="C11:C13"/>
     <mergeCell ref="C14:C15"/>
@@ -2357,14 +2373,11 @@
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="B4:B8"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="A27:A36"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="K34:K36"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A37:A40"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="A17:A26"/>
+    <mergeCell ref="A3:A16"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="B22:B25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2582,7 +2595,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="87" x14ac:dyDescent="0.35">
-      <c r="A22" s="30" t="s">
+      <c r="A22" s="25" t="s">
         <v>111</v>
       </c>
       <c r="B22" s="2" t="s">
@@ -2596,7 +2609,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="30"/>
+      <c r="A23" s="25"/>
       <c r="B23" s="2" t="s">
         <v>122</v>
       </c>
@@ -2608,8 +2621,8 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="30"/>
-      <c r="B24" s="30" t="s">
+      <c r="A24" s="25"/>
+      <c r="B24" s="25" t="s">
         <v>122</v>
       </c>
       <c r="C24" s="15">
@@ -2623,8 +2636,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A25" s="30"/>
-      <c r="B25" s="30"/>
+      <c r="A25" s="25"/>
+      <c r="B25" s="25"/>
       <c r="C25" s="15">
         <v>45820</v>
       </c>
@@ -2633,8 +2646,8 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A26" s="30"/>
-      <c r="B26" s="30"/>
+      <c r="A26" s="25"/>
+      <c r="B26" s="25"/>
       <c r="C26" s="15">
         <v>45820</v>
       </c>
@@ -2643,8 +2656,8 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="333.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="30"/>
-      <c r="B27" s="30" t="s">
+      <c r="A27" s="25"/>
+      <c r="B27" s="25" t="s">
         <v>123</v>
       </c>
       <c r="C27" s="15">
@@ -2659,7 +2672,7 @@
     </row>
     <row r="28" spans="1:5" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A28" s="20"/>
-      <c r="B28" s="30"/>
+      <c r="B28" s="25"/>
       <c r="C28" s="15">
         <v>45821</v>
       </c>
@@ -2708,7 +2721,7 @@
         <v>45836</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>